<commit_message>
lagt til ny excel fil med nett
</commit_message>
<xml_diff>
--- a/Grid/test_trøndelagsnettet.xlsx
+++ b/Grid/test_trøndelagsnettet.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/b57458e082dedb4f/Dokumenter/EMIL 1. klasse høst/TET4205 Power system analysis 2/Kraftsystemer-2/Grid/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="18" documentId="11_057EBA57FA9E57F87E476CE1F4362D3B786B1A4C" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BE75181C-1E1D-4F2E-9CF4-6554412DA2D6}"/>
+  <xr:revisionPtr revIDLastSave="25" documentId="11_057EBA57FA9E57F87E476CE1F4362D3B786B1A4C" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BE410DF7-B8CF-4B1F-92A6-3E640775DBB2}"/>
   <bookViews>
-    <workbookView xWindow="754" yWindow="754" windowWidth="18515" windowHeight="10740" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-103" yWindow="-103" windowWidth="24892" windowHeight="14914" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="bus" sheetId="1" r:id="rId1"/>
@@ -776,6 +776,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1065,6 +1069,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:M22"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <cols>
+    <col min="7" max="7" width="17.921875" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
@@ -5039,6 +5046,8 @@
   <dimension ref="A1:M19"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
+    <col min="9" max="9" width="11.3046875" customWidth="1"/>
+    <col min="10" max="10" width="13.23046875" customWidth="1"/>
     <col min="12" max="12" width="0" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -5788,6 +5797,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:G5"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <cols>
+    <col min="1" max="1" width="22.3828125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">

</xml_diff>

<commit_message>
La inn et god oversiktark som kan sjekke N-1 kriteritet ordentlig
</commit_message>
<xml_diff>
--- a/Grid/test_trøndelagsnettet.xlsx
+++ b/Grid/test_trøndelagsnettet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0348cbc925570652/Master/Kraftsystemer/Kraftsystemer-2/Grid/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3" documentId="11_D66F0DED9A5C76CD19CE15FAE4E891D83F9B944B" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{68021297-1237-4FD7-B733-4D36A35FCEB3}"/>
+  <xr:revisionPtr revIDLastSave="52" documentId="11_D66F0DED9A5C76CD19CE15FAE4E891D83F9B944B" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2DEEC584-BFA7-4AA5-B31D-6DAC1B173902}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="484" uniqueCount="223">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="487" uniqueCount="224">
   <si>
     <t>line_id</t>
   </si>
@@ -330,12 +330,6 @@
     <t>bus</t>
   </si>
   <si>
-    <t>Unnamed: 9</t>
-  </si>
-  <si>
-    <t>Unnamed: 10</t>
-  </si>
-  <si>
     <t>Grytten</t>
   </si>
   <si>
@@ -706,6 +700,15 @@
   </si>
   <si>
     <t>B_per_m</t>
+  </si>
+  <si>
+    <t>S_max</t>
+  </si>
+  <si>
+    <t>V_max</t>
+  </si>
+  <si>
+    <t>V_min</t>
   </si>
 </sst>
 </file>
@@ -775,7 +778,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -784,6 +787,8 @@
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -799,6 +804,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1086,10 +1095,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:M22"/>
+  <dimension ref="A1:P22"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>65</v>
       </c>
@@ -1129,8 +1138,17 @@
       <c r="M1" s="1" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N1" s="1" t="s">
+        <v>221</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>222</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="2" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>30</v>
       </c>
@@ -1162,7 +1180,7 @@
         <v>100</v>
       </c>
       <c r="K2">
-        <f t="shared" ref="K2:K22" si="0">0.25*J2</f>
+        <f>0.25*J2</f>
         <v>25</v>
       </c>
       <c r="L2">
@@ -1171,8 +1189,17 @@
       <c r="M2">
         <v>30</v>
       </c>
-    </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N2">
+        <v>1200</v>
+      </c>
+      <c r="O2" s="5">
+        <v>1.2</v>
+      </c>
+      <c r="P2">
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="3" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>45</v>
       </c>
@@ -1201,20 +1228,29 @@
         <v>0</v>
       </c>
       <c r="J3" s="3">
-        <v>300</v>
+        <v>200</v>
       </c>
       <c r="K3">
-        <f t="shared" si="0"/>
-        <v>75</v>
+        <f t="shared" ref="K3:K22" si="0">0.25*J3</f>
+        <v>50</v>
       </c>
       <c r="L3">
-        <v>1150</v>
+        <v>0</v>
       </c>
       <c r="M3">
         <v>90</v>
       </c>
-    </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N3">
+        <v>1200</v>
+      </c>
+      <c r="O3" s="5">
+        <v>1.2</v>
+      </c>
+      <c r="P3">
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="4" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>46</v>
       </c>
@@ -1255,8 +1291,17 @@
       <c r="M4">
         <v>0</v>
       </c>
-    </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N4">
+        <v>1200</v>
+      </c>
+      <c r="O4" s="5">
+        <v>1.2</v>
+      </c>
+      <c r="P4">
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="5" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>60</v>
       </c>
@@ -1297,8 +1342,17 @@
       <c r="M5">
         <v>0</v>
       </c>
-    </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N5">
+        <v>1200</v>
+      </c>
+      <c r="O5" s="5">
+        <v>1.2</v>
+      </c>
+      <c r="P5">
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="6" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A6">
         <v>61</v>
       </c>
@@ -1339,8 +1393,17 @@
       <c r="M6">
         <v>0</v>
       </c>
-    </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N6">
+        <v>1200</v>
+      </c>
+      <c r="O6" s="5">
+        <v>1.2</v>
+      </c>
+      <c r="P6">
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="7" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A7">
         <v>62</v>
       </c>
@@ -1381,8 +1444,17 @@
       <c r="M7">
         <v>30</v>
       </c>
-    </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N7">
+        <v>1200</v>
+      </c>
+      <c r="O7" s="5">
+        <v>1.2</v>
+      </c>
+      <c r="P7">
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="8" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A8">
         <v>76</v>
       </c>
@@ -1423,8 +1495,17 @@
       <c r="M8">
         <v>15</v>
       </c>
-    </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N8">
+        <v>1200</v>
+      </c>
+      <c r="O8" s="5">
+        <v>1.2</v>
+      </c>
+      <c r="P8">
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="9" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A9">
         <v>77</v>
       </c>
@@ -1465,8 +1546,17 @@
       <c r="M9">
         <v>15</v>
       </c>
-    </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N9">
+        <v>1200</v>
+      </c>
+      <c r="O9" s="5">
+        <v>1.2</v>
+      </c>
+      <c r="P9">
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="10" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A10">
         <v>78</v>
       </c>
@@ -1507,8 +1597,17 @@
       <c r="M10">
         <v>0</v>
       </c>
-    </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N10">
+        <v>1200</v>
+      </c>
+      <c r="O10" s="5">
+        <v>1.2</v>
+      </c>
+      <c r="P10">
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="11" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A11">
         <v>79</v>
       </c>
@@ -1549,8 +1648,17 @@
       <c r="M11">
         <v>60</v>
       </c>
-    </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N11">
+        <v>1200</v>
+      </c>
+      <c r="O11" s="5">
+        <v>1.2</v>
+      </c>
+      <c r="P11">
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="12" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A12">
         <v>80</v>
       </c>
@@ -1579,11 +1687,11 @@
         <v>0</v>
       </c>
       <c r="J12" s="3">
-        <v>150</v>
+        <v>200</v>
       </c>
       <c r="K12">
         <f t="shared" si="0"/>
-        <v>37.5</v>
+        <v>50</v>
       </c>
       <c r="L12">
         <v>40</v>
@@ -1591,8 +1699,17 @@
       <c r="M12">
         <v>45</v>
       </c>
-    </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N12">
+        <v>1200</v>
+      </c>
+      <c r="O12" s="5">
+        <v>1.2</v>
+      </c>
+      <c r="P12">
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="13" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A13">
         <v>105</v>
       </c>
@@ -1621,11 +1738,11 @@
         <v>0</v>
       </c>
       <c r="J13" s="3">
-        <v>50</v>
+        <v>500</v>
       </c>
       <c r="K13">
         <f t="shared" si="0"/>
-        <v>12.5</v>
+        <v>125</v>
       </c>
       <c r="L13">
         <v>330</v>
@@ -1633,8 +1750,17 @@
       <c r="M13">
         <v>15</v>
       </c>
-    </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N13">
+        <v>1200</v>
+      </c>
+      <c r="O13" s="5">
+        <v>1.2</v>
+      </c>
+      <c r="P13">
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="14" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A14">
         <v>106</v>
       </c>
@@ -1675,8 +1801,17 @@
       <c r="M14">
         <v>75</v>
       </c>
-    </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N14">
+        <v>1200</v>
+      </c>
+      <c r="O14" s="5">
+        <v>1.2</v>
+      </c>
+      <c r="P14">
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="15" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A15">
         <v>107</v>
       </c>
@@ -1717,8 +1852,17 @@
       <c r="M15">
         <v>0</v>
       </c>
-    </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N15">
+        <v>1200</v>
+      </c>
+      <c r="O15" s="5">
+        <v>1.2</v>
+      </c>
+      <c r="P15">
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="16" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A16">
         <v>108</v>
       </c>
@@ -1757,10 +1901,19 @@
         <v>70</v>
       </c>
       <c r="M16">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.35">
+        <v>400</v>
+      </c>
+      <c r="N16">
+        <v>1200</v>
+      </c>
+      <c r="O16" s="5">
+        <v>1.2</v>
+      </c>
+      <c r="P16">
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="17" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A17">
         <v>109</v>
       </c>
@@ -1801,8 +1954,17 @@
       <c r="M17">
         <v>15</v>
       </c>
-    </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N17">
+        <v>1200</v>
+      </c>
+      <c r="O17" s="5">
+        <v>1.2</v>
+      </c>
+      <c r="P17">
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="18" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A18">
         <v>138</v>
       </c>
@@ -1843,8 +2005,17 @@
       <c r="M18">
         <v>30</v>
       </c>
-    </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N18">
+        <v>1200</v>
+      </c>
+      <c r="O18" s="5">
+        <v>1.2</v>
+      </c>
+      <c r="P18">
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="19" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A19">
         <v>139</v>
       </c>
@@ -1885,8 +2056,17 @@
       <c r="M19">
         <v>45</v>
       </c>
-    </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N19">
+        <v>1200</v>
+      </c>
+      <c r="O19" s="5">
+        <v>1.2</v>
+      </c>
+      <c r="P19">
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="20" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A20">
         <v>141</v>
       </c>
@@ -1927,8 +2107,17 @@
       <c r="M20">
         <v>135</v>
       </c>
-    </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N20">
+        <v>1200</v>
+      </c>
+      <c r="O20" s="5">
+        <v>1.2</v>
+      </c>
+      <c r="P20">
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="21" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A21">
         <v>161</v>
       </c>
@@ -1969,8 +2158,17 @@
       <c r="M21">
         <v>165</v>
       </c>
-    </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N21">
+        <v>1200</v>
+      </c>
+      <c r="O21" s="5">
+        <v>1.2</v>
+      </c>
+      <c r="P21">
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="22" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A22">
         <v>176</v>
       </c>
@@ -2010,6 +2208,15 @@
       </c>
       <c r="M22">
         <v>30</v>
+      </c>
+      <c r="N22">
+        <v>1200</v>
+      </c>
+      <c r="O22" s="5">
+        <v>1.2</v>
+      </c>
+      <c r="P22">
+        <v>0.7</v>
       </c>
     </row>
   </sheetData>
@@ -2019,10 +2226,10 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:K105"/>
+  <dimension ref="A1:I105"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>8</v>
       </c>
@@ -2050,22 +2257,16 @@
       <c r="I1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="J1" s="1" t="s">
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
         <v>97</v>
       </c>
-      <c r="K1" s="1" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
+      <c r="B2" t="s">
+        <v>98</v>
+      </c>
+      <c r="C2" t="s">
         <v>99</v>
-      </c>
-      <c r="B2" t="s">
-        <v>100</v>
-      </c>
-      <c r="C2" t="s">
-        <v>101</v>
       </c>
       <c r="D2">
         <v>143</v>
@@ -2086,15 +2287,15 @@
         <v>8.8044759999999993</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="B3" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C3" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="D3">
         <v>60</v>
@@ -2115,15 +2316,15 @@
         <v>11.871930600000001</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="B4" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C4" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="D4">
         <v>251</v>
@@ -2144,15 +2345,15 @@
         <v>5.2955095999999999</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="B5" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C5" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="D5">
         <v>160</v>
@@ -2173,15 +2374,15 @@
         <v>8.8866494000000031</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="B6" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C6" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="D6">
         <v>92</v>
@@ -2202,15 +2403,15 @@
         <v>10.0126685</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="B7" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C7" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="D7">
         <v>14</v>
@@ -2231,15 +2432,15 @@
         <v>11.08352</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="B8" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C8" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="D8">
         <v>140</v>
@@ -2260,15 +2461,15 @@
         <v>10.481959399999999</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="B9" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C9" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="D9">
         <v>157.30000000000001</v>
@@ -2289,15 +2490,15 @@
         <v>5.6666667000000004</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="B10" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C10" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="D10">
         <v>259.8</v>
@@ -2318,15 +2519,15 @@
         <v>11.1900113</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="B11" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C11" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="D11">
         <v>46</v>
@@ -2347,15 +2548,15 @@
         <v>11.0058121</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="B12" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C12" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="D12">
         <v>9</v>
@@ -2376,15 +2577,15 @@
         <v>12.458487</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="B13" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C13" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="D13">
         <v>100</v>
@@ -2405,15 +2606,15 @@
         <v>5.9323598000000004</v>
       </c>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="B14" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C14" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D14">
         <v>5.4</v>
@@ -2434,15 +2635,15 @@
         <v>12.426399999999999</v>
       </c>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="B15" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C15" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D15">
         <v>109</v>
@@ -2463,15 +2664,15 @@
         <v>8.0306999999999995</v>
       </c>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
+        <v>115</v>
+      </c>
+      <c r="B16" t="s">
+        <v>116</v>
+      </c>
+      <c r="C16" t="s">
         <v>117</v>
-      </c>
-      <c r="B16" t="s">
-        <v>118</v>
-      </c>
-      <c r="C16" t="s">
-        <v>119</v>
       </c>
       <c r="D16">
         <v>253.2</v>
@@ -2494,13 +2695,13 @@
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="B17" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C17" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D17">
         <v>9</v>
@@ -2523,13 +2724,13 @@
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="B18" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C18" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D18">
         <v>169.2</v>
@@ -2552,13 +2753,13 @@
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="B19" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C19" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D19">
         <v>90</v>
@@ -2581,13 +2782,13 @@
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="B20" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C20" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D20">
         <v>26</v>
@@ -2610,13 +2811,13 @@
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="B21" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C21" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D21">
         <v>40.299999999999997</v>
@@ -2639,13 +2840,13 @@
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="B22" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C22" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D22">
         <v>6</v>
@@ -2668,13 +2869,13 @@
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="B23" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C23" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D23">
         <v>6.2</v>
@@ -2697,13 +2898,13 @@
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B24" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C24" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D24">
         <v>14</v>
@@ -2726,13 +2927,13 @@
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="B25" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C25" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D25">
         <v>8</v>
@@ -2755,13 +2956,13 @@
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="B26" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C26" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D26">
         <v>48.5</v>
@@ -2784,13 +2985,13 @@
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="B27" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C27" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D27">
         <v>85</v>
@@ -2813,13 +3014,13 @@
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="B28" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C28" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D28">
         <v>5.4</v>
@@ -2842,13 +3043,13 @@
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="B29" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C29" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="D29">
         <v>9</v>
@@ -2871,13 +3072,13 @@
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="B30" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C30" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D30">
         <v>45</v>
@@ -2900,13 +3101,13 @@
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="B31" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C31" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D31">
         <v>86</v>
@@ -2929,13 +3130,13 @@
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="B32" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C32" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D32">
         <v>64</v>
@@ -2958,13 +3159,13 @@
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="B33" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C33" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="D33">
         <v>319.2</v>
@@ -2987,13 +3188,13 @@
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="B34" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C34" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="D34">
         <v>23</v>
@@ -3016,13 +3217,13 @@
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="B35" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C35" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D35">
         <v>60</v>
@@ -3045,13 +3246,13 @@
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="B36" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C36" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D36">
         <v>36</v>
@@ -3074,13 +3275,13 @@
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="B37" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C37" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D37">
         <v>3</v>
@@ -3103,13 +3304,13 @@
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="B38" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C38" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D38">
         <v>70</v>
@@ -3132,13 +3333,13 @@
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="B39" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C39" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D39">
         <v>19.5</v>
@@ -3161,13 +3362,13 @@
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="B40" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C40" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D40">
         <v>7.8</v>
@@ -3190,13 +3391,13 @@
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="B41" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C41" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D41">
         <v>5.8</v>
@@ -3219,13 +3420,13 @@
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="B42" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C42" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D42">
         <v>8</v>
@@ -3248,13 +3449,13 @@
     </row>
     <row r="43" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="B43" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C43" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D43">
         <v>17</v>
@@ -3277,13 +3478,13 @@
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="B44" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C44" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D44">
         <v>25.2</v>
@@ -3306,13 +3507,13 @@
     </row>
     <row r="45" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="B45" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C45" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D45">
         <v>4.0999999999999996</v>
@@ -3335,13 +3536,13 @@
     </row>
     <row r="46" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="B46" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C46" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D46">
         <v>4</v>
@@ -3364,13 +3565,13 @@
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="B47" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C47" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D47">
         <v>2</v>
@@ -3393,13 +3594,13 @@
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="B48" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C48" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D48">
         <v>10.4</v>
@@ -3422,13 +3623,13 @@
     </row>
     <row r="49" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="B49" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C49" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D49">
         <v>100</v>
@@ -3451,13 +3652,13 @@
     </row>
     <row r="50" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="B50" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C50" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D50">
         <v>21.7</v>
@@ -3480,13 +3681,13 @@
     </row>
     <row r="51" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="B51" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C51" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D51">
         <v>5.2</v>
@@ -3509,13 +3710,13 @@
     </row>
     <row r="52" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="B52" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C52" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D52">
         <v>5.4</v>
@@ -3538,13 +3739,13 @@
     </row>
     <row r="53" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="B53" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C53" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D53">
         <v>9</v>
@@ -3567,13 +3768,13 @@
     </row>
     <row r="54" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="B54" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C54" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D54">
         <v>5.5</v>
@@ -3596,13 +3797,13 @@
     </row>
     <row r="55" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="B55" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C55" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D55">
         <v>10.6</v>
@@ -3625,13 +3826,13 @@
     </row>
     <row r="56" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="B56" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C56" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D56">
         <v>11.5</v>
@@ -3654,13 +3855,13 @@
     </row>
     <row r="57" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="B57" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C57" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D57">
         <v>40</v>
@@ -3683,13 +3884,13 @@
     </row>
     <row r="58" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="B58" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C58" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D58">
         <v>35</v>
@@ -3712,13 +3913,13 @@
     </row>
     <row r="59" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="B59" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C59" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D59">
         <v>9</v>
@@ -3741,13 +3942,13 @@
     </row>
     <row r="60" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="B60" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C60" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D60">
         <v>16.3</v>
@@ -3770,13 +3971,13 @@
     </row>
     <row r="61" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="B61" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C61" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D61">
         <v>45</v>
@@ -3799,13 +4000,13 @@
     </row>
     <row r="62" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="B62" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C62" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D62">
         <v>8</v>
@@ -3828,13 +4029,13 @@
     </row>
     <row r="63" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="B63" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C63" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D63">
         <v>4.5999999999999996</v>
@@ -3857,13 +4058,13 @@
     </row>
     <row r="64" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="B64" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C64" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D64">
         <v>10</v>
@@ -3886,13 +4087,13 @@
     </row>
     <row r="65" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="B65" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C65" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D65">
         <v>36.6</v>
@@ -3915,13 +4116,13 @@
     </row>
     <row r="66" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A66" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="B66" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C66" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D66">
         <v>5</v>
@@ -3944,13 +4145,13 @@
     </row>
     <row r="67" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="B67" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C67" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D67">
         <v>3.7</v>
@@ -3973,13 +4174,13 @@
     </row>
     <row r="68" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A68" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="B68" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C68" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D68">
         <v>5.7</v>
@@ -4002,13 +4203,13 @@
     </row>
     <row r="69" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A69" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="B69" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C69" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D69">
         <v>5.6</v>
@@ -4031,13 +4232,13 @@
     </row>
     <row r="70" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A70" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="B70" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C70" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D70">
         <v>2</v>
@@ -4060,13 +4261,13 @@
     </row>
     <row r="71" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="B71" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C71" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D71">
         <v>12</v>
@@ -4089,13 +4290,13 @@
     </row>
     <row r="72" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="B72" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="C72" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="D72">
         <v>37.5</v>
@@ -4118,13 +4319,13 @@
     </row>
     <row r="73" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A73" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="B73" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C73" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D73">
         <v>16</v>
@@ -4147,13 +4348,13 @@
     </row>
     <row r="74" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A74" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="B74" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C74" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D74">
         <v>108</v>
@@ -4176,13 +4377,13 @@
     </row>
     <row r="75" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A75" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="B75" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C75" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D75">
         <v>28</v>
@@ -4205,13 +4406,13 @@
     </row>
     <row r="76" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A76" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="B76" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C76" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D76">
         <v>5</v>
@@ -4234,13 +4435,13 @@
     </row>
     <row r="77" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A77" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="B77" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C77" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D77">
         <v>9.5</v>
@@ -4263,13 +4464,13 @@
     </row>
     <row r="78" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A78" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="B78" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C78" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="D78">
         <v>30</v>
@@ -4292,13 +4493,13 @@
     </row>
     <row r="79" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A79" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="B79" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C79" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="D79">
         <v>130</v>
@@ -4321,13 +4522,13 @@
     </row>
     <row r="80" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A80" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="B80" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C80" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D80">
         <v>1.5</v>
@@ -4350,13 +4551,13 @@
     </row>
     <row r="81" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A81" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="B81" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C81" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D81">
         <v>3.5</v>
@@ -4379,13 +4580,13 @@
     </row>
     <row r="82" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A82" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="B82" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C82" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D82">
         <v>4.4000000000000004</v>
@@ -4408,13 +4609,13 @@
     </row>
     <row r="83" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A83" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="B83" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C83" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D83">
         <v>0.3</v>
@@ -4437,13 +4638,13 @@
     </row>
     <row r="84" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A84" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="B84" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C84" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D84">
         <v>8.1999999999999993</v>
@@ -4466,13 +4667,13 @@
     </row>
     <row r="85" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A85" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="B85" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C85" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D85">
         <v>4.8</v>
@@ -4495,13 +4696,13 @@
     </row>
     <row r="86" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A86" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="B86" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C86" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D86">
         <v>8.1</v>
@@ -4524,13 +4725,13 @@
     </row>
     <row r="87" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A87" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="B87" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C87" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D87">
         <v>5.5</v>
@@ -4553,13 +4754,13 @@
     </row>
     <row r="88" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A88" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="B88" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C88" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D88">
         <v>40</v>
@@ -4582,13 +4783,13 @@
     </row>
     <row r="89" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A89" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="B89" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C89" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D89">
         <v>0.4</v>
@@ -4611,13 +4812,13 @@
     </row>
     <row r="90" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A90" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="B90" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C90" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D90">
         <v>2</v>
@@ -4640,13 +4841,13 @@
     </row>
     <row r="91" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A91" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="B91" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C91" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D91">
         <v>105</v>
@@ -4669,13 +4870,13 @@
     </row>
     <row r="92" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A92" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="B92" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C92" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D92">
         <v>4.8</v>
@@ -4698,13 +4899,13 @@
     </row>
     <row r="93" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A93" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="B93" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C93" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D93">
         <v>2.4</v>
@@ -4727,13 +4928,13 @@
     </row>
     <row r="94" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A94" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="B94" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C94" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D94">
         <v>12.7</v>
@@ -4756,13 +4957,13 @@
     </row>
     <row r="95" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A95" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="B95" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C95" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D95">
         <v>12.7</v>
@@ -4785,13 +4986,13 @@
     </row>
     <row r="96" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A96" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="B96" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C96" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D96">
         <v>3</v>
@@ -4814,13 +5015,13 @@
     </row>
     <row r="97" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A97" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="B97" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C97" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D97">
         <v>13.7</v>
@@ -4843,13 +5044,13 @@
     </row>
     <row r="98" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A98" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="B98" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C98" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D98">
         <v>41</v>
@@ -4872,13 +5073,13 @@
     </row>
     <row r="99" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A99" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="B99" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C99" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D99">
         <v>1.3</v>
@@ -4901,13 +5102,13 @@
     </row>
     <row r="100" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A100" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="B100" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="C100" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="D100">
         <v>31</v>
@@ -4930,13 +5131,13 @@
     </row>
     <row r="101" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A101" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="B101" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C101" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D101">
         <v>6.5</v>
@@ -4959,13 +5160,13 @@
     </row>
     <row r="102" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A102" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="B102" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C102" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D102">
         <v>23.9</v>
@@ -4988,13 +5189,13 @@
     </row>
     <row r="103" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A103" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="B103" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C103" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D103">
         <v>8.4</v>
@@ -5017,13 +5218,13 @@
     </row>
     <row r="104" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A104" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="B104" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C104" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D104">
         <v>3.2</v>
@@ -5046,13 +5247,13 @@
     </row>
     <row r="105" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A105" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="B105" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C105" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D105">
         <v>5.5</v>
@@ -5080,13 +5281,13 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:M19"/>
+  <dimension ref="A1:N19"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="12" max="12" width="13" hidden="1" customWidth="1"/>
+    <col min="12" max="12" width="1.36328125" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -5112,13 +5313,13 @@
         <v>7</v>
       </c>
       <c r="I1" s="1" t="s">
+        <v>218</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>219</v>
+      </c>
+      <c r="K1" s="1" t="s">
         <v>220</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>221</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>222</v>
       </c>
       <c r="L1" s="1" t="s">
         <v>8</v>
@@ -5126,8 +5327,11 @@
       <c r="M1" s="1" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N1" s="1" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>1166</v>
       </c>
@@ -5167,8 +5371,11 @@
       <c r="M2">
         <v>10943</v>
       </c>
-    </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N2">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>1334</v>
       </c>
@@ -5208,8 +5415,11 @@
       <c r="M3" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N3">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>1335</v>
       </c>
@@ -5246,8 +5456,11 @@
       <c r="L4" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N4">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>1336</v>
       </c>
@@ -5287,8 +5500,11 @@
       <c r="M5">
         <v>3343</v>
       </c>
-    </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N5">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A6">
         <v>1165</v>
       </c>
@@ -5325,8 +5541,11 @@
       <c r="L6" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N6">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A7">
         <v>1289</v>
       </c>
@@ -5363,8 +5582,11 @@
       <c r="L7" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N7">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A8">
         <v>1290</v>
       </c>
@@ -5404,8 +5626,11 @@
       <c r="M8">
         <v>343321</v>
       </c>
-    </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N8">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A9">
         <v>1291</v>
       </c>
@@ -5442,8 +5667,11 @@
       <c r="L9" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N9">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A10">
         <v>1173</v>
       </c>
@@ -5480,8 +5708,11 @@
       <c r="L10" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N10">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A11">
         <v>1174</v>
       </c>
@@ -5518,8 +5749,11 @@
       <c r="L11" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N11">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A12">
         <v>1292</v>
       </c>
@@ -5556,8 +5790,11 @@
       <c r="L12" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N12">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="13" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A13">
         <v>1175</v>
       </c>
@@ -5594,8 +5831,11 @@
       <c r="L13" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N13">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="14" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A14">
         <v>6798</v>
       </c>
@@ -5632,8 +5872,11 @@
       <c r="L14" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N14">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="15" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A15">
         <v>1288</v>
       </c>
@@ -5670,8 +5913,11 @@
       <c r="L15" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N15">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="16" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A16">
         <v>6562</v>
       </c>
@@ -5708,8 +5954,11 @@
       <c r="L16" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="N16">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="17" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A17">
         <v>1293</v>
       </c>
@@ -5746,8 +5995,11 @@
       <c r="L17" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="N17">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="18" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A18">
         <v>1176</v>
       </c>
@@ -5784,8 +6036,11 @@
       <c r="L18" t="s">
         <v>61</v>
       </c>
-    </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="N18">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="19" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A19">
         <v>1317</v>
       </c>
@@ -5821,6 +6076,9 @@
       </c>
       <c r="L19" t="s">
         <v>64</v>
+      </c>
+      <c r="N19">
+        <v>600</v>
       </c>
     </row>
   </sheetData>
@@ -5830,12 +6088,15 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="7" max="7" width="0" hidden="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>2</v>
@@ -5844,19 +6105,22 @@
         <v>3</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>208</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>209</v>
+      </c>
+      <c r="F1" s="1" t="s">
         <v>210</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>211</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>212</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="H1" s="1" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>43</v>
       </c>
@@ -5876,10 +6140,13 @@
         <v>2.8000000000000001E-2</v>
       </c>
       <c r="G2" t="s">
-        <v>213</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
+        <v>211</v>
+      </c>
+      <c r="H2" s="4">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>44</v>
       </c>
@@ -5899,10 +6166,13 @@
         <v>0.04</v>
       </c>
       <c r="G3" t="s">
-        <v>214</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
+        <v>212</v>
+      </c>
+      <c r="H3" s="4">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>45</v>
       </c>
@@ -5922,10 +6192,13 @@
         <v>2.8000000000000001E-2</v>
       </c>
       <c r="G4" t="s">
-        <v>215</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
+        <v>213</v>
+      </c>
+      <c r="H4" s="4">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>46</v>
       </c>
@@ -5945,7 +6218,10 @@
         <v>2.8000000000000001E-2</v>
       </c>
       <c r="G5" t="s">
-        <v>216</v>
+        <v>214</v>
+      </c>
+      <c r="H5" s="4">
+        <v>300</v>
       </c>
     </row>
   </sheetData>
@@ -5960,7 +6236,7 @@
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>8</v>
@@ -5969,7 +6245,7 @@
         <v>1</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>2</v>
@@ -5984,7 +6260,7 @@
         <v>7</v>
       </c>
       <c r="I1" s="2" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
     </row>
   </sheetData>

</xml_diff>